<commit_message>
Phase 3: persistent research unlocks for all structures
Add data-driven structure unlocks (smelter, conveyor-fast, assembler /
miner-advanced stubs), ResearchState with paid confirm unlocks, Italian
Ricerca UI, and build-menu gating. Persist unlocked IDs in save v3
(with Phase 1–2 migration). Extend --self-test for locked start,
unlock spend, and reload retention.

Co-authored-by: Gianni Nacu <Juan0177@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/game-data.xlsx
+++ b/data/game-data.xlsx
@@ -8,10 +8,12 @@
   <x:sheets>
     <x:sheet name="Conveyors" sheetId="1" r:id="rId2"/>
     <x:sheet name="Recipes" sheetId="2" r:id="rId3"/>
+    <x:sheet name="Structures" sheetId="3" r:id="rId4"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Conveyors!$A$1:$I$3</x:definedName>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Recipes!$A$1:$D$2</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Structures!$A$1:$G$7</x:definedName>
   </x:definedNames>
   <x:calcPr calcId="125725"/>
 </x:workbook>
@@ -78,6 +80,66 @@
   </x:si>
   <x:si>
     <x:t>iron-ore:2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DisplayName</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Kind</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UnlockedByDefault</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IsStub</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nastro base</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Conveyor</x:t>
+  </x:si>
+  <x:si>
+    <x:t>miner</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Minatore</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Building</x:t>
+  </x:si>
+  <x:si>
+    <x:t>smelter</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Forno</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nastro veloce</x:t>
+  </x:si>
+  <x:si>
+    <x:t>assembler</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Assemblatore</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Stub</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:30;copper-wire:10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>miner-advanced</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Minatore avanzato</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:25</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -609,4 +671,192 @@
   <x:headerFooter/>
   <x:tableParts count="0"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:G7"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="15.424911" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18.139196" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="9.567768" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18.139196" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13.567768" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="26.282054" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="6.424911" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:7" s="1" customFormat="1">
+      <x:c r="A1" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G1" s="1" t="s">
+        <x:v>23</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:7">
+      <x:c r="A2" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:7">
+      <x:c r="A3" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E3" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:7">
+      <x:c r="A4" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="0">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:7">
+      <x:c r="A5" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="0">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:7">
+      <x:c r="A6" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="0">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:7">
+      <x:c r="A7" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="0">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:autoFilter ref="A1:G7"/>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Phase 4: content-driven market, wallet UI, core upgrade sinks
Sell prices and building costs come from content; session ledger tracks
gain/loss; core upgrade adds a money sink; Italian market panel shows
reinvestment hint; economy state persists in save v4.

Co-authored-by: Gianni Nacu <Juan0177@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/game-data.xlsx
+++ b/data/game-data.xlsx
@@ -9,11 +9,17 @@
     <x:sheet name="Conveyors" sheetId="1" r:id="rId2"/>
     <x:sheet name="Recipes" sheetId="2" r:id="rId3"/>
     <x:sheet name="Structures" sheetId="3" r:id="rId4"/>
+    <x:sheet name="Market" sheetId="4" r:id="rId5"/>
+    <x:sheet name="Buildings" sheetId="5" r:id="rId6"/>
+    <x:sheet name="Economy" sheetId="6" r:id="rId7"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Conveyors!$A$1:$I$3</x:definedName>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Recipes!$A$1:$D$2</x:definedName>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Structures!$A$1:$G$7</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Market!$A$1:$C$4</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Buildings!$A$1:$D$3</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Economy!$A$1:$D$2</x:definedName>
   </x:definedNames>
   <x:calcPr calcId="125725"/>
 </x:workbook>
@@ -140,6 +146,57 @@
   </x:si>
   <x:si>
     <x:t>iron-plate:25</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ItemId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SellPrice</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-ore</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ferro grezzo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Lastra di ferro</x:t>
+  </x:si>
+  <x:si>
+    <x:t>copper-wire</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Filo di rame</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RefundPercent</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CoreUpgradeMoney</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CoreUpgradeMaterials</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SaleBonusPercent</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RefundPolicyNote</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Rimozione edifici/nastri: rimborso completo (100%).</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -859,4 +916,189 @@
   <x:headerFooter/>
   <x:tableParts count="0"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:C4"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="11.424911" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.282054" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8.282054" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:3" s="1" customFormat="1">
+      <x:c r="A1" s="1" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:3">
+      <x:c r="A2" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="C2" s="0">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:3">
+      <x:c r="A3" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="C3" s="0">
+        <x:v>30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:3">
+      <x:c r="A4" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="C4" s="0">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:autoFilter ref="A1:C4"/>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:D3"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="7.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.282054" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11.139196" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14.282054" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:4" s="1" customFormat="1">
+      <x:c r="A1" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="s">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:4">
+      <x:c r="A2" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B2" s="0">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D2" s="0">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:4">
+      <x:c r="A3" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B3" s="0">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D3" s="0">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:autoFilter ref="A1:D3"/>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:D2"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="19.282054" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="21.139196" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16.996339" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="47.282054" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:4" s="1" customFormat="1">
+      <x:c r="A1" s="1" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="s">
+        <x:v>54</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:4">
+      <x:c r="A2" s="0">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="C2" s="0">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:autoFilter ref="A1:D2"/>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Phase 5: self-tests for copper, branching, bridge, assembler
Junction pass-through fix; Excel content sync; stress handoff on long
belt lines; save v5 coverage for assemblers and bridges.

Co-authored-by: Gianni Nacu <Juan0177@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/game-data.xlsx
+++ b/data/game-data.xlsx
@@ -14,11 +14,11 @@
     <x:sheet name="Economy" sheetId="6" r:id="rId7"/>
   </x:sheets>
   <x:definedNames>
-    <x:definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Conveyors!$A$1:$I$3</x:definedName>
-    <x:definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Recipes!$A$1:$D$2</x:definedName>
-    <x:definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Structures!$A$1:$G$7</x:definedName>
-    <x:definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Market!$A$1:$C$4</x:definedName>
-    <x:definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Buildings!$A$1:$D$3</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Conveyors!$A$1:$J$6</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Recipes!$A$1:$D$3</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Structures!$A$1:$G$10</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Market!$A$1:$C$5</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Buildings!$A$1:$D$4</x:definedName>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Economy!$A$1:$D$2</x:definedName>
   </x:definedNames>
   <x:calcPr calcId="125725"/>
@@ -55,6 +55,9 @@
     <x:t>UnlockMaterials</x:t>
   </x:si>
   <x:si>
+    <x:t>Kind</x:t>
+  </x:si>
+  <x:si>
     <x:t>conveyor-basic</x:t>
   </x:si>
   <x:si>
@@ -64,6 +67,9 @@
     <x:t/>
   </x:si>
   <x:si>
+    <x:t>belt</x:t>
+  </x:si>
+  <x:si>
     <x:t>conveyor-fast</x:t>
   </x:si>
   <x:si>
@@ -73,6 +79,36 @@
     <x:t>iron-plate:50</x:t>
   </x:si>
   <x:si>
+    <x:t>junction</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>splitter</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>conveyor-bridge</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:3;copper-wire:1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>bridge</x:t>
+  </x:si>
+  <x:si>
     <x:t>DurationSeconds</x:t>
   </x:si>
   <x:si>
@@ -88,12 +124,18 @@
     <x:t>iron-ore:2</x:t>
   </x:si>
   <x:si>
+    <x:t>craft-copper-wire</x:t>
+  </x:si>
+  <x:si>
+    <x:t>copper-ore:1;iron-plate:1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>copper-wire:2</x:t>
+  </x:si>
+  <x:si>
     <x:t>DisplayName</x:t>
   </x:si>
   <x:si>
-    <x:t>Kind</x:t>
-  </x:si>
-  <x:si>
     <x:t>UnlockedByDefault</x:t>
   </x:si>
   <x:si>
@@ -121,30 +163,36 @@
     <x:t>Forno</x:t>
   </x:si>
   <x:si>
-    <x:t>iron-plate:15</x:t>
-  </x:si>
-  <x:si>
     <x:t>Nastro veloce</x:t>
   </x:si>
   <x:si>
+    <x:t>Incrocio</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sdoppiatore</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nastro ponte</x:t>
+  </x:si>
+  <x:si>
     <x:t>assembler</x:t>
   </x:si>
   <x:si>
     <x:t>Assemblatore</x:t>
   </x:si>
   <x:si>
+    <x:t>iron-plate:25;copper-wire:5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>miner-advanced</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Minatore avanzato</x:t>
+  </x:si>
+  <x:si>
     <x:t>Stub</x:t>
   </x:si>
   <x:si>
-    <x:t>iron-plate:30;copper-wire:10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>miner-advanced</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Minatore avanzato</x:t>
-  </x:si>
-  <x:si>
     <x:t>iron-plate:25</x:t>
   </x:si>
   <x:si>
@@ -166,6 +214,12 @@
     <x:t>Lastra di ferro</x:t>
   </x:si>
   <x:si>
+    <x:t>copper-ore</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Rame grezzo</x:t>
+  </x:si>
+  <x:si>
     <x:t>copper-wire</x:t>
   </x:si>
   <x:si>
@@ -181,6 +235,9 @@
     <x:t>iron-plate:6</x:t>
   </x:si>
   <x:si>
+    <x:t>iron-plate:8;copper-wire:2</x:t>
+  </x:si>
+  <x:si>
     <x:t>CoreUpgradeMoney</x:t>
   </x:si>
   <x:si>
@@ -191,9 +248,6 @@
   </x:si>
   <x:si>
     <x:t>RefundPolicyNote</x:t>
-  </x:si>
-  <x:si>
-    <x:t>iron-plate:20</x:t>
   </x:si>
   <x:si>
     <x:t>Rimozione edifici/nastri: rimborso completo (100%).</x:t>
@@ -567,10 +621,10 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:I3"/>
+  <x:dimension ref="A1:J6"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14.424911" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15.567768" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="4.139196" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="19.710625" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="8.567768" style="0" customWidth="1"/>
@@ -579,9 +633,10 @@
     <x:col min="7" max="7" width="24.282054" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="13.567768" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="15.424911" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="8.424911" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:9" s="1" customFormat="1">
+    <x:row r="1" spans="1:10" s="1" customFormat="1">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -609,10 +664,13 @@
       <x:c r="I1" s="1" t="s">
         <x:v>8</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:9">
+      <x:c r="J1" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:10">
       <x:c r="A2" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0">
         <x:v>1</x:v>
@@ -630,18 +688,21 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H2" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:9">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J2" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:10">
       <x:c r="A3" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B3" s="0">
         <x:v>2</x:v>
@@ -659,17 +720,116 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H3" s="0">
         <x:v>250</x:v>
       </x:c>
       <x:c r="I3" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J3" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:10">
+      <x:c r="A4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B4" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C4" s="0">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="D4" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E4" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F4" s="0">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="H4" s="0">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="I4" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:10">
+      <x:c r="A5" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B5" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" s="0">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="D5" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E5" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F5" s="0">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="H5" s="0">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="I5" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="J5" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:10">
+      <x:c r="A6" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B6" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="0">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D6" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F6" s="0">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H6" s="0">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="I6" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="J6" s="0" t="s">
+        <x:v>26</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:autoFilter ref="A1:I3"/>
+  <x:autoFilter ref="A1:J6"/>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
@@ -683,13 +843,13 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D2"/>
+  <x:dimension ref="A1:D3"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16.139196" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="16.282054" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="9.710625" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="11.139196" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23.567768" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13.282054" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:4" s="1" customFormat="1">
@@ -697,31 +857,45 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>15</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4">
       <x:c r="A2" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B2" s="0">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:4">
+      <x:c r="A3" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B3" s="0">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>34</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:autoFilter ref="A1:D2"/>
+  <x:autoFilter ref="A1:D3"/>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
@@ -735,15 +909,15 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:G7"/>
+  <x:dimension ref="A1:G10"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="15.424911" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15.567768" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="18.139196" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="9.567768" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="18.139196" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="13.567768" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="26.282054" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25.282054" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="6.424911" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -752,13 +926,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E1" s="1" t="s">
         <x:v>7</x:v>
@@ -767,18 +941,18 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G1" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>37</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:7">
       <x:c r="A2" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D2" s="0" t="b">
         <x:v>1</x:v>
@@ -787,7 +961,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G2" s="0" t="b">
         <x:v>0</x:v>
@@ -795,13 +969,13 @@
     </x:row>
     <x:row r="3" spans="1:7">
       <x:c r="A3" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D3" s="0" t="b">
         <x:v>1</x:v>
@@ -810,7 +984,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G3" s="0" t="b">
         <x:v>0</x:v>
@@ -818,13 +992,13 @@
     </x:row>
     <x:row r="4" spans="1:7">
       <x:c r="A4" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D4" s="0" t="b">
         <x:v>0</x:v>
@@ -833,7 +1007,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="G4" s="0" t="b">
         <x:v>0</x:v>
@@ -841,13 +1015,13 @@
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="A5" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D5" s="0" t="b">
         <x:v>0</x:v>
@@ -856,7 +1030,7 @@
         <x:v>250</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G5" s="0" t="b">
         <x:v>0</x:v>
@@ -864,52 +1038,121 @@
     </x:row>
     <x:row r="6" spans="1:7">
       <x:c r="A6" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D6" s="0" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>400</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G6" s="0" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:7">
       <x:c r="A7" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D7" s="0" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="0">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:7">
+      <x:c r="A8" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="0">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G8" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:7">
+      <x:c r="A9" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="0">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G9" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:7">
+      <x:c r="A10" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="0">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="F7" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="G7" s="0" t="b">
+      <x:c r="F10" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="G10" s="0" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:autoFilter ref="A1:G7"/>
+  <x:autoFilter ref="A1:G10"/>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
@@ -923,7 +1166,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C4"/>
+  <x:dimension ref="A1:C5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="11.424911" style="0" customWidth="1"/>
@@ -933,21 +1176,21 @@
   <x:sheetData>
     <x:row r="1" spans="1:3" s="1" customFormat="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>41</x:v>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C2" s="0">
         <x:v>8</x:v>
@@ -955,10 +1198,10 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C3" s="0">
         <x:v>30</x:v>
@@ -966,17 +1209,28 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C4" s="0">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:3">
+      <x:c r="A5" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="C5" s="0">
         <x:v>14</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:autoFilter ref="A1:C4"/>
+  <x:autoFilter ref="A1:C5"/>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
@@ -990,12 +1244,12 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D3"/>
+  <x:dimension ref="A1:D4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="7.710625" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="11.282054" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="11.139196" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24.282054" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="14.282054" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -1010,18 +1264,18 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>48</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4">
       <x:c r="A2" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B2" s="0">
         <x:v>25</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D2" s="0">
         <x:v>100</x:v>
@@ -1029,20 +1283,34 @@
     </x:row>
     <x:row r="3" spans="1:4">
       <x:c r="A3" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B3" s="0">
         <x:v>40</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D3" s="0">
         <x:v>100</x:v>
       </x:c>
     </x:row>
+    <x:row r="4" spans="1:4">
+      <x:c r="A4" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B4" s="0">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D4" s="0">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:autoFilter ref="A1:D3"/>
+  <x:autoFilter ref="A1:D4"/>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
@@ -1067,16 +1335,16 @@
   <x:sheetData>
     <x:row r="1" spans="1:4" s="1" customFormat="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>51</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>52</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>53</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>54</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4">
@@ -1084,13 +1352,13 @@
         <x:v>150</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C2" s="0">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Phase 6: power stub, seed select, onboarding, polish
Core+generator power budget gates crafting; New Game seed scenarios;
contextual Italian tips; save v6; belt handoff perf; balance tweaks.

Co-authored-by: Gianni Nacu <Juan0177@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/game-data.xlsx
+++ b/data/game-data.xlsx
@@ -16,9 +16,9 @@
   <x:definedNames>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Conveyors!$A$1:$J$6</x:definedName>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Recipes!$A$1:$D$3</x:definedName>
-    <x:definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Structures!$A$1:$G$10</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Structures!$A$1:$G$11</x:definedName>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Market!$A$1:$C$5</x:definedName>
-    <x:definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Buildings!$A$1:$D$4</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Buildings!$A$1:$D$5</x:definedName>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Economy!$A$1:$D$2</x:definedName>
   </x:definedNames>
   <x:calcPr calcId="125725"/>
@@ -181,7 +181,16 @@
     <x:t>Assemblatore</x:t>
   </x:si>
   <x:si>
-    <x:t>iron-plate:25;copper-wire:5</x:t>
+    <x:t>iron-plate:22;copper-wire:4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>generator</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Generatore</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:12</x:t>
   </x:si>
   <x:si>
     <x:t>miner-advanced</x:t>
@@ -236,6 +245,9 @@
   </x:si>
   <x:si>
     <x:t>iron-plate:8;copper-wire:2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>iron-plate:8</x:t>
   </x:si>
   <x:si>
     <x:t>CoreUpgradeMoney</x:t>
@@ -909,7 +921,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:G10"/>
+  <x:dimension ref="A1:G11"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="15.567768" style="0" customWidth="1"/>
@@ -1119,7 +1131,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="0">
-        <x:v>250</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="F9" s="0" t="s">
         <x:v>51</x:v>
@@ -1136,23 +1148,46 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="0">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="F10" s="0" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="D10" s="0" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E10" s="0">
+      <x:c r="G10" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:7">
+      <x:c r="A11" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="0">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="F10" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="G10" s="0" t="b">
+      <x:c r="F11" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="G11" s="0" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:autoFilter ref="A1:G10"/>
+  <x:autoFilter ref="A1:G11"/>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
@@ -1176,21 +1211,21 @@
   <x:sheetData>
     <x:row r="1" spans="1:3" s="1" customFormat="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>56</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
         <x:v>35</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>57</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C2" s="0">
         <x:v>8</x:v>
@@ -1198,10 +1233,10 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C3" s="0">
         <x:v>30</x:v>
@@ -1209,10 +1244,10 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C4" s="0">
         <x:v>6</x:v>
@@ -1220,13 +1255,13 @@
     </x:row>
     <x:row r="5" spans="1:3">
       <x:c r="A5" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C5" s="0">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1244,7 +1279,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D4"/>
+  <x:dimension ref="A1:D5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
@@ -1264,7 +1299,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4">
@@ -1275,7 +1310,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D2" s="0">
         <x:v>100</x:v>
@@ -1289,7 +1324,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="D3" s="0">
         <x:v>100</x:v>
@@ -1303,14 +1338,28 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D4" s="0">
         <x:v>100</x:v>
       </x:c>
     </x:row>
+    <x:row r="5" spans="1:4">
+      <x:c r="A5" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B5" s="0">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D5" s="0">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:autoFilter ref="A1:D4"/>
+  <x:autoFilter ref="A1:D5"/>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
@@ -1335,16 +1384,16 @@
   <x:sheetData>
     <x:row r="1" spans="1:4" s="1" customFormat="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>70</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>73</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4">
@@ -1358,7 +1407,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>